<commit_message>
Modified Domain entities to include explicit references to the Student entity.
</commit_message>
<xml_diff>
--- a/MetaEdOutput/Documentation/DataDictionary/XmlDataDictionary.xlsx
+++ b/MetaEdOutput/Documentation/DataDictionary/XmlDataDictionary.xlsx
@@ -45312,7 +45312,7 @@
         <v>2970</v>
       </c>
       <c r="C1924" t="s">
-        <v>61</v>
+        <v>1460</v>
       </c>
       <c r="D1924" t="s">
         <v>8</v>
@@ -45329,7 +45329,7 @@
         <v>2970</v>
       </c>
       <c r="C1925" t="s">
-        <v>966</v>
+        <v>1388</v>
       </c>
       <c r="D1925" t="s">
         <v>8</v>
@@ -45346,7 +45346,7 @@
         <v>2970</v>
       </c>
       <c r="C1926" t="s">
-        <v>1581</v>
+        <v>452</v>
       </c>
       <c r="D1926" t="s">
         <v>8</v>
@@ -45363,7 +45363,7 @@
         <v>2970</v>
       </c>
       <c r="C1927" t="s">
-        <v>1178</v>
+        <v>61</v>
       </c>
       <c r="D1927" t="s">
         <v>8</v>
@@ -45380,7 +45380,7 @@
         <v>2970</v>
       </c>
       <c r="C1928" t="s">
-        <v>1631</v>
+        <v>966</v>
       </c>
       <c r="D1928" t="s">
         <v>8</v>
@@ -45397,7 +45397,7 @@
         <v>2970</v>
       </c>
       <c r="C1929" t="s">
-        <v>1598</v>
+        <v>1581</v>
       </c>
       <c r="D1929" t="s">
         <v>8</v>
@@ -45414,7 +45414,7 @@
         <v>2970</v>
       </c>
       <c r="C1930" t="s">
-        <v>1632</v>
+        <v>1178</v>
       </c>
       <c r="D1930" t="s">
         <v>8</v>
@@ -45425,801 +45425,801 @@
     </row>
     <row r="1931">
       <c r="A1931" t="s">
-        <v>3027</v>
+        <v>3003</v>
       </c>
       <c r="B1931" t="s">
-        <v>1287</v>
+        <v>2970</v>
       </c>
       <c r="C1931" t="s">
-        <v>3028</v>
+        <v>1608</v>
       </c>
       <c r="D1931" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E1931" t="s">
-        <v>3029</v>
+        <v>3021</v>
       </c>
     </row>
     <row r="1932">
       <c r="A1932" t="s">
-        <v>3030</v>
+        <v>3003</v>
       </c>
       <c r="B1932" t="s">
-        <v>3028</v>
+        <v>2970</v>
       </c>
       <c r="C1932" t="s">
-        <v>225</v>
+        <v>1619</v>
       </c>
       <c r="D1932" t="s">
         <v>8</v>
       </c>
       <c r="E1932" t="s">
-        <v>3031</v>
+        <v>3021</v>
       </c>
     </row>
     <row r="1933">
       <c r="A1933" t="s">
-        <v>3032</v>
+        <v>3003</v>
       </c>
       <c r="B1933" t="s">
-        <v>368</v>
+        <v>2970</v>
       </c>
       <c r="C1933" t="s">
-        <v>3033</v>
+        <v>1624</v>
       </c>
       <c r="D1933" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E1933" t="s">
-        <v>3034</v>
+        <v>3021</v>
       </c>
     </row>
     <row r="1934">
       <c r="A1934" t="s">
-        <v>3035</v>
+        <v>3003</v>
       </c>
       <c r="B1934" t="s">
-        <v>443</v>
+        <v>2970</v>
       </c>
       <c r="C1934" t="s">
-        <v>3036</v>
+        <v>1631</v>
       </c>
       <c r="D1934" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E1934" t="s">
-        <v>3037</v>
+        <v>3021</v>
       </c>
     </row>
     <row r="1935">
       <c r="A1935" t="s">
-        <v>3038</v>
+        <v>3003</v>
       </c>
       <c r="B1935" t="s">
-        <v>444</v>
+        <v>2970</v>
       </c>
       <c r="C1935" t="s">
-        <v>3039</v>
+        <v>1598</v>
       </c>
       <c r="D1935" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E1935" t="s">
-        <v>3040</v>
+        <v>3021</v>
       </c>
     </row>
     <row r="1936">
       <c r="A1936" t="s">
-        <v>3041</v>
+        <v>3003</v>
       </c>
       <c r="B1936" t="s">
-        <v>445</v>
+        <v>2970</v>
       </c>
       <c r="C1936" t="s">
-        <v>3042</v>
+        <v>1632</v>
       </c>
       <c r="D1936" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E1936" t="s">
-        <v>3043</v>
+        <v>3021</v>
       </c>
     </row>
     <row r="1937">
       <c r="A1937" t="s">
-        <v>3044</v>
+        <v>3027</v>
       </c>
       <c r="B1937" t="s">
-        <v>3042</v>
+        <v>1287</v>
       </c>
       <c r="C1937" t="s">
-        <v>875</v>
+        <v>3028</v>
       </c>
       <c r="D1937" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E1937" t="s">
-        <v>3045</v>
+        <v>3029</v>
       </c>
     </row>
     <row r="1938">
       <c r="A1938" t="s">
-        <v>3044</v>
+        <v>3030</v>
       </c>
       <c r="B1938" t="s">
-        <v>3042</v>
+        <v>3028</v>
       </c>
       <c r="C1938" t="s">
-        <v>677</v>
+        <v>225</v>
       </c>
       <c r="D1938" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="E1938" t="s">
-        <v>3046</v>
+        <v>3031</v>
       </c>
     </row>
     <row r="1939">
       <c r="A1939" t="s">
-        <v>3044</v>
+        <v>3032</v>
       </c>
       <c r="B1939" t="s">
-        <v>3042</v>
+        <v>368</v>
       </c>
       <c r="C1939" t="s">
-        <v>1467</v>
+        <v>3033</v>
       </c>
       <c r="D1939" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E1939" t="s">
-        <v>3045</v>
+        <v>3034</v>
       </c>
     </row>
     <row r="1940">
       <c r="A1940" t="s">
-        <v>3047</v>
+        <v>3035</v>
       </c>
       <c r="B1940" t="s">
-        <v>369</v>
+        <v>443</v>
       </c>
       <c r="C1940" t="s">
-        <v>3048</v>
+        <v>3036</v>
       </c>
       <c r="D1940" t="s">
         <v>13</v>
       </c>
       <c r="E1940" t="s">
-        <v>3049</v>
+        <v>3037</v>
       </c>
     </row>
     <row r="1941">
       <c r="A1941" t="s">
-        <v>3050</v>
+        <v>3038</v>
       </c>
       <c r="B1941" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="C1941" t="s">
-        <v>3051</v>
+        <v>3039</v>
       </c>
       <c r="D1941" t="s">
         <v>13</v>
       </c>
       <c r="E1941" t="s">
-        <v>3052</v>
+        <v>3040</v>
       </c>
     </row>
     <row r="1942">
       <c r="A1942" t="s">
-        <v>3053</v>
+        <v>3041</v>
       </c>
       <c r="B1942" t="s">
-        <v>697</v>
+        <v>445</v>
       </c>
       <c r="C1942" t="s">
-        <v>3054</v>
+        <v>3042</v>
       </c>
       <c r="D1942" t="s">
         <v>13</v>
       </c>
       <c r="E1942" t="s">
-        <v>3055</v>
+        <v>3043</v>
       </c>
     </row>
     <row r="1943">
       <c r="A1943" t="s">
-        <v>3056</v>
+        <v>3044</v>
       </c>
       <c r="B1943" t="s">
-        <v>447</v>
+        <v>3042</v>
       </c>
       <c r="C1943" t="s">
-        <v>3057</v>
+        <v>875</v>
       </c>
       <c r="D1943" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E1943" t="s">
-        <v>3058</v>
+        <v>3045</v>
       </c>
     </row>
     <row r="1944">
       <c r="A1944" t="s">
-        <v>3059</v>
+        <v>3044</v>
       </c>
       <c r="B1944" t="s">
-        <v>3026</v>
+        <v>3042</v>
       </c>
       <c r="C1944" t="s">
-        <v>3060</v>
+        <v>677</v>
       </c>
       <c r="D1944" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E1944" t="s">
-        <v>3061</v>
+        <v>3046</v>
       </c>
     </row>
     <row r="1945">
       <c r="A1945" t="s">
-        <v>3062</v>
+        <v>3044</v>
       </c>
       <c r="B1945" t="s">
-        <v>719</v>
+        <v>3042</v>
       </c>
       <c r="C1945" t="s">
-        <v>476</v>
+        <v>1467</v>
       </c>
       <c r="D1945" t="s">
         <v>8</v>
       </c>
       <c r="E1945" t="s">
-        <v>3063</v>
+        <v>3045</v>
       </c>
     </row>
     <row r="1946">
       <c r="A1946" t="s">
-        <v>3062</v>
+        <v>3047</v>
       </c>
       <c r="B1946" t="s">
-        <v>719</v>
+        <v>369</v>
       </c>
       <c r="C1946" t="s">
-        <v>2969</v>
+        <v>3048</v>
       </c>
       <c r="D1946" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E1946" t="s">
-        <v>3063</v>
+        <v>3049</v>
       </c>
     </row>
     <row r="1947">
       <c r="A1947" t="s">
-        <v>3062</v>
+        <v>3050</v>
       </c>
       <c r="B1947" t="s">
-        <v>719</v>
+        <v>446</v>
       </c>
       <c r="C1947" t="s">
-        <v>478</v>
+        <v>3051</v>
       </c>
       <c r="D1947" t="s">
         <v>13</v>
       </c>
       <c r="E1947" t="s">
-        <v>3063</v>
+        <v>3052</v>
       </c>
     </row>
     <row r="1948">
       <c r="A1948" t="s">
-        <v>3064</v>
+        <v>3053</v>
       </c>
       <c r="B1948" t="s">
-        <v>3065</v>
+        <v>697</v>
       </c>
       <c r="C1948" t="s">
-        <v>347</v>
+        <v>3054</v>
       </c>
       <c r="D1948" t="s">
         <v>13</v>
       </c>
       <c r="E1948" t="s">
-        <v>3066</v>
+        <v>3055</v>
       </c>
     </row>
     <row r="1949">
       <c r="A1949" t="s">
-        <v>3067</v>
+        <v>3056</v>
       </c>
       <c r="B1949" t="s">
-        <v>64</v>
+        <v>447</v>
       </c>
       <c r="C1949" t="s">
-        <v>405</v>
+        <v>3057</v>
       </c>
       <c r="D1949" t="s">
         <v>13</v>
       </c>
       <c r="E1949" t="s">
-        <v>3068</v>
+        <v>3058</v>
       </c>
     </row>
     <row r="1950">
       <c r="A1950" t="s">
-        <v>3069</v>
+        <v>3059</v>
       </c>
       <c r="B1950" t="s">
-        <v>866</v>
+        <v>3026</v>
       </c>
       <c r="C1950" t="s">
-        <v>681</v>
+        <v>3060</v>
       </c>
       <c r="D1950" t="s">
         <v>13</v>
       </c>
       <c r="E1950" t="s">
-        <v>3070</v>
+        <v>3061</v>
       </c>
     </row>
     <row r="1951">
       <c r="A1951" t="s">
-        <v>3069</v>
+        <v>3062</v>
       </c>
       <c r="B1951" t="s">
-        <v>866</v>
+        <v>719</v>
       </c>
       <c r="C1951" t="s">
-        <v>35</v>
+        <v>476</v>
       </c>
       <c r="D1951" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E1951" t="s">
-        <v>3071</v>
+        <v>3063</v>
       </c>
     </row>
     <row r="1952">
       <c r="A1952" t="s">
-        <v>3072</v>
+        <v>3062</v>
       </c>
       <c r="B1952" t="s">
-        <v>647</v>
+        <v>719</v>
       </c>
       <c r="C1952" t="s">
-        <v>1144</v>
+        <v>2969</v>
       </c>
       <c r="D1952" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E1952" t="s">
-        <v>3073</v>
+        <v>3063</v>
       </c>
     </row>
     <row r="1953">
       <c r="A1953" t="s">
-        <v>3074</v>
+        <v>3062</v>
       </c>
       <c r="B1953" t="s">
-        <v>1216</v>
+        <v>719</v>
       </c>
       <c r="C1953" t="s">
-        <v>1144</v>
+        <v>478</v>
       </c>
       <c r="D1953" t="s">
         <v>13</v>
       </c>
       <c r="E1953" t="s">
-        <v>3075</v>
+        <v>3063</v>
       </c>
     </row>
     <row r="1954">
       <c r="A1954" t="s">
-        <v>3076</v>
+        <v>3064</v>
       </c>
       <c r="B1954" t="s">
-        <v>1316</v>
+        <v>3065</v>
       </c>
       <c r="C1954" t="s">
-        <v>1144</v>
+        <v>347</v>
       </c>
       <c r="D1954" t="s">
         <v>13</v>
       </c>
       <c r="E1954" t="s">
-        <v>3077</v>
+        <v>3066</v>
       </c>
     </row>
     <row r="1955">
       <c r="A1955" t="s">
-        <v>3078</v>
+        <v>3067</v>
       </c>
       <c r="B1955" t="s">
-        <v>175</v>
+        <v>64</v>
       </c>
       <c r="C1955" t="s">
-        <v>1424</v>
+        <v>405</v>
       </c>
       <c r="D1955" t="s">
         <v>13</v>
       </c>
       <c r="E1955" t="s">
-        <v>3079</v>
+        <v>3068</v>
       </c>
     </row>
     <row r="1956">
       <c r="A1956" t="s">
-        <v>3080</v>
+        <v>3069</v>
       </c>
       <c r="B1956" t="s">
-        <v>175</v>
+        <v>866</v>
       </c>
       <c r="C1956" t="s">
-        <v>1424</v>
+        <v>681</v>
       </c>
       <c r="D1956" t="s">
         <v>13</v>
       </c>
       <c r="E1956" t="s">
-        <v>3081</v>
+        <v>3070</v>
       </c>
     </row>
     <row r="1957">
       <c r="A1957" t="s">
-        <v>3082</v>
+        <v>3069</v>
       </c>
       <c r="B1957" t="s">
-        <v>3083</v>
+        <v>866</v>
       </c>
       <c r="C1957" t="s">
-        <v>121</v>
+        <v>35</v>
       </c>
       <c r="D1957" t="s">
         <v>13</v>
       </c>
       <c r="E1957" t="s">
-        <v>3084</v>
+        <v>3071</v>
       </c>
     </row>
     <row r="1958">
       <c r="A1958" t="s">
-        <v>3085</v>
+        <v>3072</v>
       </c>
       <c r="B1958" t="s">
-        <v>3086</v>
+        <v>647</v>
       </c>
       <c r="C1958" t="s">
-        <v>1146</v>
+        <v>1144</v>
       </c>
       <c r="D1958" t="s">
         <v>13</v>
       </c>
       <c r="E1958" t="s">
-        <v>3087</v>
+        <v>3073</v>
       </c>
     </row>
     <row r="1959">
       <c r="A1959" t="s">
-        <v>3088</v>
+        <v>3074</v>
       </c>
       <c r="B1959" t="s">
-        <v>798</v>
+        <v>1216</v>
       </c>
       <c r="C1959" t="s">
-        <v>3089</v>
+        <v>1144</v>
       </c>
       <c r="D1959" t="s">
         <v>13</v>
       </c>
       <c r="E1959" t="s">
-        <v>3090</v>
+        <v>3075</v>
       </c>
     </row>
     <row r="1960">
       <c r="A1960" t="s">
-        <v>3091</v>
+        <v>3076</v>
       </c>
       <c r="B1960" t="s">
-        <v>269</v>
+        <v>1316</v>
       </c>
       <c r="C1960" t="s">
-        <v>1146</v>
+        <v>1144</v>
       </c>
       <c r="D1960" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E1960" t="s">
-        <v>3092</v>
+        <v>3077</v>
       </c>
     </row>
     <row r="1961">
       <c r="A1961" t="s">
-        <v>3091</v>
+        <v>3078</v>
       </c>
       <c r="B1961" t="s">
-        <v>269</v>
+        <v>175</v>
       </c>
       <c r="C1961" t="s">
-        <v>2037</v>
+        <v>1424</v>
       </c>
       <c r="D1961" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E1961" t="s">
-        <v>3092</v>
+        <v>3079</v>
       </c>
     </row>
     <row r="1962">
       <c r="A1962" t="s">
-        <v>3093</v>
+        <v>3080</v>
       </c>
       <c r="B1962" t="s">
-        <v>2037</v>
+        <v>175</v>
       </c>
       <c r="C1962" t="s">
-        <v>3094</v>
+        <v>1424</v>
       </c>
       <c r="D1962" t="s">
         <v>13</v>
       </c>
       <c r="E1962" t="s">
-        <v>3095</v>
+        <v>3081</v>
       </c>
     </row>
     <row r="1963">
       <c r="A1963" t="s">
-        <v>3096</v>
+        <v>3082</v>
       </c>
       <c r="B1963" t="s">
-        <v>3097</v>
+        <v>3083</v>
       </c>
       <c r="C1963" t="s">
-        <v>706</v>
+        <v>121</v>
       </c>
       <c r="D1963" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E1963" t="s">
-        <v>3098</v>
+        <v>3084</v>
       </c>
     </row>
     <row r="1964">
       <c r="A1964" t="s">
-        <v>3099</v>
+        <v>3085</v>
       </c>
       <c r="B1964" t="s">
-        <v>2371</v>
+        <v>3086</v>
       </c>
       <c r="C1964" t="s">
-        <v>3100</v>
+        <v>1146</v>
       </c>
       <c r="D1964" t="s">
         <v>13</v>
       </c>
       <c r="E1964" t="s">
-        <v>3101</v>
+        <v>3087</v>
       </c>
     </row>
     <row r="1965">
       <c r="A1965" t="s">
-        <v>3102</v>
+        <v>3088</v>
       </c>
       <c r="B1965" t="s">
-        <v>2423</v>
+        <v>798</v>
       </c>
       <c r="C1965" t="s">
-        <v>3103</v>
+        <v>3089</v>
       </c>
       <c r="D1965" t="s">
         <v>13</v>
       </c>
       <c r="E1965" t="s">
-        <v>3104</v>
+        <v>3090</v>
       </c>
     </row>
     <row r="1966">
       <c r="A1966" t="s">
-        <v>1946</v>
+        <v>3091</v>
       </c>
       <c r="B1966" t="s">
-        <v>1946</v>
+        <v>269</v>
       </c>
       <c r="C1966" t="s">
-        <v>648</v>
+        <v>1146</v>
       </c>
       <c r="D1966" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="E1966" t="s">
-        <v>3105</v>
+        <v>3092</v>
       </c>
     </row>
     <row r="1967">
       <c r="A1967" t="s">
-        <v>3106</v>
+        <v>3091</v>
       </c>
       <c r="B1967" t="s">
-        <v>3103</v>
+        <v>269</v>
       </c>
       <c r="C1967" t="s">
-        <v>648</v>
+        <v>2037</v>
       </c>
       <c r="D1967" t="s">
         <v>8</v>
       </c>
       <c r="E1967" t="s">
-        <v>2422</v>
+        <v>3092</v>
       </c>
     </row>
     <row r="1968">
       <c r="A1968" t="s">
-        <v>3106</v>
+        <v>3093</v>
       </c>
       <c r="B1968" t="s">
-        <v>3103</v>
+        <v>2037</v>
       </c>
       <c r="C1968" t="s">
-        <v>3107</v>
+        <v>3094</v>
       </c>
       <c r="D1968" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E1968" t="s">
-        <v>2422</v>
+        <v>3095</v>
       </c>
     </row>
     <row r="1969">
       <c r="A1969" t="s">
-        <v>3108</v>
+        <v>3096</v>
       </c>
       <c r="B1969" t="s">
-        <v>3107</v>
+        <v>3097</v>
       </c>
       <c r="C1969" t="s">
-        <v>3109</v>
+        <v>706</v>
       </c>
       <c r="D1969" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E1969" t="s">
-        <v>3110</v>
+        <v>3098</v>
       </c>
     </row>
     <row r="1970">
       <c r="A1970" t="s">
-        <v>2078</v>
+        <v>3099</v>
       </c>
       <c r="B1970" t="s">
-        <v>2078</v>
+        <v>2371</v>
       </c>
       <c r="C1970" t="s">
-        <v>648</v>
+        <v>3100</v>
       </c>
       <c r="D1970" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E1970" t="s">
-        <v>3111</v>
+        <v>3101</v>
       </c>
     </row>
     <row r="1971">
       <c r="A1971" t="s">
-        <v>3112</v>
+        <v>3102</v>
       </c>
       <c r="B1971" t="s">
-        <v>222</v>
+        <v>2423</v>
       </c>
       <c r="C1971" t="s">
-        <v>2078</v>
+        <v>3103</v>
       </c>
       <c r="D1971" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E1971" t="s">
-        <v>3113</v>
+        <v>3104</v>
       </c>
     </row>
     <row r="1972">
       <c r="A1972" t="s">
-        <v>3114</v>
+        <v>1946</v>
       </c>
       <c r="B1972" t="s">
-        <v>3094</v>
+        <v>1946</v>
       </c>
       <c r="C1972" t="s">
-        <v>1942</v>
+        <v>648</v>
       </c>
       <c r="D1972" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="E1972" t="s">
-        <v>3115</v>
+        <v>3105</v>
       </c>
     </row>
     <row r="1973">
       <c r="A1973" t="s">
-        <v>3114</v>
+        <v>3106</v>
       </c>
       <c r="B1973" t="s">
-        <v>3094</v>
+        <v>3103</v>
       </c>
       <c r="C1973" t="s">
-        <v>706</v>
+        <v>648</v>
       </c>
       <c r="D1973" t="s">
         <v>8</v>
       </c>
       <c r="E1973" t="s">
-        <v>3116</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="1974">
       <c r="A1974" t="s">
-        <v>3114</v>
+        <v>3106</v>
       </c>
       <c r="B1974" t="s">
-        <v>3094</v>
+        <v>3103</v>
       </c>
       <c r="C1974" t="s">
-        <v>3117</v>
+        <v>3107</v>
       </c>
       <c r="D1974" t="s">
         <v>8</v>
       </c>
       <c r="E1974" t="s">
-        <v>3115</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="1975">
       <c r="A1975" t="s">
-        <v>3114</v>
+        <v>3108</v>
       </c>
       <c r="B1975" t="s">
-        <v>3094</v>
+        <v>3107</v>
       </c>
       <c r="C1975" t="s">
-        <v>796</v>
+        <v>3109</v>
       </c>
       <c r="D1975" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E1975" t="s">
-        <v>3118</v>
+        <v>3110</v>
       </c>
     </row>
     <row r="1976">
       <c r="A1976" t="s">
-        <v>3114</v>
+        <v>2078</v>
       </c>
       <c r="B1976" t="s">
-        <v>3094</v>
+        <v>2078</v>
       </c>
       <c r="C1976" t="s">
-        <v>2369</v>
+        <v>648</v>
       </c>
       <c r="D1976" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="E1976" t="s">
-        <v>3118</v>
+        <v>3111</v>
       </c>
     </row>
     <row r="1977">
       <c r="A1977" t="s">
-        <v>3114</v>
+        <v>3112</v>
       </c>
       <c r="B1977" t="s">
-        <v>3094</v>
+        <v>222</v>
       </c>
       <c r="C1977" t="s">
-        <v>2665</v>
+        <v>2078</v>
       </c>
       <c r="D1977" t="s">
         <v>8</v>
       </c>
       <c r="E1977" t="s">
-        <v>3119</v>
+        <v>3113</v>
       </c>
     </row>
     <row r="1978">
@@ -46230,13 +46230,13 @@
         <v>3094</v>
       </c>
       <c r="C1978" t="s">
-        <v>798</v>
+        <v>1942</v>
       </c>
       <c r="D1978" t="s">
         <v>8</v>
       </c>
       <c r="E1978" t="s">
-        <v>3118</v>
+        <v>3115</v>
       </c>
     </row>
     <row r="1979">
@@ -46247,13 +46247,13 @@
         <v>3094</v>
       </c>
       <c r="C1979" t="s">
-        <v>2371</v>
+        <v>706</v>
       </c>
       <c r="D1979" t="s">
         <v>8</v>
       </c>
       <c r="E1979" t="s">
-        <v>3118</v>
+        <v>3116</v>
       </c>
     </row>
     <row r="1980">
@@ -46264,7 +46264,7 @@
         <v>3094</v>
       </c>
       <c r="C1980" t="s">
-        <v>2423</v>
+        <v>3117</v>
       </c>
       <c r="D1980" t="s">
         <v>8</v>
@@ -46281,13 +46281,13 @@
         <v>3094</v>
       </c>
       <c r="C1981" t="s">
-        <v>3120</v>
+        <v>796</v>
       </c>
       <c r="D1981" t="s">
         <v>8</v>
       </c>
       <c r="E1981" t="s">
-        <v>3116</v>
+        <v>3118</v>
       </c>
     </row>
     <row r="1982">
@@ -46298,13 +46298,13 @@
         <v>3094</v>
       </c>
       <c r="C1982" t="s">
-        <v>2667</v>
+        <v>2369</v>
       </c>
       <c r="D1982" t="s">
         <v>8</v>
       </c>
       <c r="E1982" t="s">
-        <v>3119</v>
+        <v>3118</v>
       </c>
     </row>
     <row r="1983">
@@ -46315,183 +46315,183 @@
         <v>3094</v>
       </c>
       <c r="C1983" t="s">
-        <v>3121</v>
+        <v>2665</v>
       </c>
       <c r="D1983" t="s">
         <v>8</v>
       </c>
       <c r="E1983" t="s">
-        <v>3115</v>
+        <v>3119</v>
       </c>
     </row>
     <row r="1984">
       <c r="A1984" t="s">
-        <v>3122</v>
+        <v>3114</v>
       </c>
       <c r="B1984" t="s">
-        <v>1174</v>
+        <v>3094</v>
       </c>
       <c r="C1984" t="s">
-        <v>3123</v>
+        <v>798</v>
       </c>
       <c r="D1984" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E1984" t="s">
-        <v>3124</v>
+        <v>3118</v>
       </c>
     </row>
     <row r="1985">
       <c r="A1985" t="s">
-        <v>3125</v>
+        <v>3114</v>
       </c>
       <c r="B1985" t="s">
-        <v>269</v>
+        <v>3094</v>
       </c>
       <c r="C1985" t="s">
-        <v>706</v>
+        <v>2371</v>
       </c>
       <c r="D1985" t="s">
         <v>8</v>
       </c>
       <c r="E1985" t="s">
-        <v>3126</v>
+        <v>3118</v>
       </c>
     </row>
     <row r="1986">
       <c r="A1986" t="s">
-        <v>3125</v>
+        <v>3114</v>
       </c>
       <c r="B1986" t="s">
-        <v>269</v>
+        <v>3094</v>
       </c>
       <c r="C1986" t="s">
-        <v>3120</v>
+        <v>2423</v>
       </c>
       <c r="D1986" t="s">
         <v>8</v>
       </c>
       <c r="E1986" t="s">
-        <v>3126</v>
+        <v>3115</v>
       </c>
     </row>
     <row r="1987">
       <c r="A1987" t="s">
-        <v>3127</v>
+        <v>3114</v>
       </c>
       <c r="B1987" t="s">
+        <v>3094</v>
+      </c>
+      <c r="C1987" t="s">
         <v>3120</v>
       </c>
-      <c r="C1987" t="s">
-        <v>3128</v>
-      </c>
       <c r="D1987" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E1987" t="s">
-        <v>3129</v>
+        <v>3116</v>
       </c>
     </row>
     <row r="1988">
       <c r="A1988" t="s">
-        <v>3130</v>
+        <v>3114</v>
       </c>
       <c r="B1988" t="s">
-        <v>3128</v>
+        <v>3094</v>
       </c>
       <c r="C1988" t="s">
-        <v>648</v>
+        <v>2667</v>
       </c>
       <c r="D1988" t="s">
         <v>8</v>
       </c>
       <c r="E1988" t="s">
-        <v>3131</v>
+        <v>3119</v>
       </c>
     </row>
     <row r="1989">
       <c r="A1989" t="s">
-        <v>3130</v>
+        <v>3114</v>
       </c>
       <c r="B1989" t="s">
-        <v>3128</v>
+        <v>3094</v>
       </c>
       <c r="C1989" t="s">
-        <v>2654</v>
+        <v>3121</v>
       </c>
       <c r="D1989" t="s">
         <v>8</v>
       </c>
       <c r="E1989" t="s">
-        <v>3131</v>
+        <v>3115</v>
       </c>
     </row>
     <row r="1990">
       <c r="A1990" t="s">
-        <v>3130</v>
+        <v>3122</v>
       </c>
       <c r="B1990" t="s">
-        <v>3128</v>
+        <v>1174</v>
       </c>
       <c r="C1990" t="s">
-        <v>1157</v>
+        <v>3123</v>
       </c>
       <c r="D1990" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E1990" t="s">
-        <v>3131</v>
+        <v>3124</v>
       </c>
     </row>
     <row r="1991">
       <c r="A1991" t="s">
-        <v>3130</v>
+        <v>3125</v>
       </c>
       <c r="B1991" t="s">
-        <v>3128</v>
+        <v>269</v>
       </c>
       <c r="C1991" t="s">
-        <v>2829</v>
+        <v>706</v>
       </c>
       <c r="D1991" t="s">
         <v>8</v>
       </c>
       <c r="E1991" t="s">
-        <v>3132</v>
+        <v>3126</v>
       </c>
     </row>
     <row r="1992">
       <c r="A1992" t="s">
-        <v>3130</v>
+        <v>3125</v>
       </c>
       <c r="B1992" t="s">
-        <v>3128</v>
+        <v>269</v>
       </c>
       <c r="C1992" t="s">
-        <v>3107</v>
+        <v>3120</v>
       </c>
       <c r="D1992" t="s">
         <v>8</v>
       </c>
       <c r="E1992" t="s">
-        <v>3131</v>
+        <v>3126</v>
       </c>
     </row>
     <row r="1993">
       <c r="A1993" t="s">
-        <v>3130</v>
+        <v>3127</v>
       </c>
       <c r="B1993" t="s">
+        <v>3120</v>
+      </c>
+      <c r="C1993" t="s">
         <v>3128</v>
       </c>
-      <c r="C1993" t="s">
-        <v>1174</v>
-      </c>
       <c r="D1993" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E1993" t="s">
-        <v>3131</v>
+        <v>3129</v>
       </c>
     </row>
     <row r="1994">
@@ -46502,13 +46502,13 @@
         <v>3128</v>
       </c>
       <c r="C1994" t="s">
-        <v>2833</v>
+        <v>648</v>
       </c>
       <c r="D1994" t="s">
         <v>8</v>
       </c>
       <c r="E1994" t="s">
-        <v>3132</v>
+        <v>3131</v>
       </c>
     </row>
     <row r="1995">
@@ -46519,7 +46519,7 @@
         <v>3128</v>
       </c>
       <c r="C1995" t="s">
-        <v>3133</v>
+        <v>2654</v>
       </c>
       <c r="D1995" t="s">
         <v>8</v>
@@ -46530,95 +46530,95 @@
     </row>
     <row r="1996">
       <c r="A1996" t="s">
-        <v>3134</v>
+        <v>3130</v>
       </c>
       <c r="B1996" t="s">
-        <v>2833</v>
+        <v>3128</v>
       </c>
       <c r="C1996" t="s">
-        <v>3135</v>
+        <v>1157</v>
       </c>
       <c r="D1996" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E1996" t="s">
-        <v>3136</v>
+        <v>3131</v>
       </c>
     </row>
     <row r="1997">
       <c r="A1997" t="s">
-        <v>3137</v>
+        <v>3130</v>
       </c>
       <c r="B1997" t="s">
-        <v>2667</v>
+        <v>3128</v>
       </c>
       <c r="C1997" t="s">
-        <v>3138</v>
+        <v>2829</v>
       </c>
       <c r="D1997" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E1997" t="s">
-        <v>3139</v>
+        <v>3132</v>
       </c>
     </row>
     <row r="1998">
       <c r="A1998" t="s">
-        <v>3140</v>
+        <v>3130</v>
       </c>
       <c r="B1998" t="s">
-        <v>3121</v>
+        <v>3128</v>
       </c>
       <c r="C1998" t="s">
-        <v>3141</v>
+        <v>3107</v>
       </c>
       <c r="D1998" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E1998" t="s">
-        <v>3142</v>
+        <v>3131</v>
       </c>
     </row>
     <row r="1999">
       <c r="A1999" t="s">
-        <v>3143</v>
+        <v>3130</v>
       </c>
       <c r="B1999" t="s">
-        <v>3141</v>
+        <v>3128</v>
       </c>
       <c r="C1999" t="s">
-        <v>1942</v>
+        <v>1174</v>
       </c>
       <c r="D1999" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E1999" t="s">
-        <v>3144</v>
+        <v>3131</v>
       </c>
     </row>
     <row r="2000">
       <c r="A2000" t="s">
-        <v>3143</v>
+        <v>3130</v>
       </c>
       <c r="B2000" t="s">
-        <v>3141</v>
+        <v>3128</v>
       </c>
       <c r="C2000" t="s">
-        <v>2654</v>
+        <v>2833</v>
       </c>
       <c r="D2000" t="s">
         <v>8</v>
       </c>
       <c r="E2000" t="s">
-        <v>3144</v>
+        <v>3132</v>
       </c>
     </row>
     <row r="2001">
       <c r="A2001" t="s">
-        <v>3143</v>
+        <v>3130</v>
       </c>
       <c r="B2001" t="s">
-        <v>3141</v>
+        <v>3128</v>
       </c>
       <c r="C2001" t="s">
         <v>3133</v>
@@ -46627,1468 +46627,1570 @@
         <v>8</v>
       </c>
       <c r="E2001" t="s">
-        <v>3144</v>
+        <v>3131</v>
       </c>
     </row>
     <row r="2002">
       <c r="A2002" t="s">
-        <v>3145</v>
+        <v>3134</v>
       </c>
       <c r="B2002" t="s">
-        <v>1175</v>
+        <v>2833</v>
       </c>
       <c r="C2002" t="s">
-        <v>3146</v>
+        <v>3135</v>
       </c>
       <c r="D2002" t="s">
         <v>13</v>
       </c>
       <c r="E2002" t="s">
-        <v>3147</v>
+        <v>3136</v>
       </c>
     </row>
     <row r="2003">
       <c r="A2003" t="s">
-        <v>3148</v>
+        <v>3137</v>
       </c>
       <c r="B2003" t="s">
-        <v>3133</v>
+        <v>2667</v>
       </c>
       <c r="C2003" t="s">
-        <v>3149</v>
+        <v>3138</v>
       </c>
       <c r="D2003" t="s">
         <v>13</v>
       </c>
       <c r="E2003" t="s">
-        <v>3150</v>
+        <v>3139</v>
       </c>
     </row>
     <row r="2004">
       <c r="A2004" t="s">
-        <v>3151</v>
+        <v>3140</v>
       </c>
       <c r="B2004" t="s">
-        <v>3149</v>
+        <v>3121</v>
       </c>
       <c r="C2004" t="s">
-        <v>1159</v>
+        <v>3141</v>
       </c>
       <c r="D2004" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E2004" t="s">
-        <v>3152</v>
+        <v>3142</v>
       </c>
     </row>
     <row r="2005">
       <c r="A2005" t="s">
-        <v>3151</v>
+        <v>3143</v>
       </c>
       <c r="B2005" t="s">
-        <v>3149</v>
+        <v>3141</v>
       </c>
       <c r="C2005" t="s">
-        <v>2831</v>
+        <v>1942</v>
       </c>
       <c r="D2005" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E2005" t="s">
-        <v>3152</v>
+        <v>3144</v>
       </c>
     </row>
     <row r="2006">
       <c r="A2006" t="s">
-        <v>3151</v>
+        <v>3143</v>
       </c>
       <c r="B2006" t="s">
-        <v>3149</v>
+        <v>3141</v>
       </c>
       <c r="C2006" t="s">
-        <v>1175</v>
+        <v>2654</v>
       </c>
       <c r="D2006" t="s">
         <v>8</v>
       </c>
       <c r="E2006" t="s">
-        <v>3152</v>
+        <v>3144</v>
       </c>
     </row>
     <row r="2007">
       <c r="A2007" t="s">
-        <v>3151</v>
+        <v>3143</v>
       </c>
       <c r="B2007" t="s">
-        <v>3149</v>
+        <v>3141</v>
       </c>
       <c r="C2007" t="s">
-        <v>2834</v>
+        <v>3133</v>
       </c>
       <c r="D2007" t="s">
         <v>8</v>
       </c>
       <c r="E2007" t="s">
-        <v>3152</v>
+        <v>3144</v>
       </c>
     </row>
     <row r="2008">
       <c r="A2008" t="s">
-        <v>3153</v>
+        <v>3145</v>
       </c>
       <c r="B2008" t="s">
-        <v>2834</v>
+        <v>1175</v>
       </c>
       <c r="C2008" t="s">
-        <v>3154</v>
+        <v>3146</v>
       </c>
       <c r="D2008" t="s">
         <v>13</v>
       </c>
       <c r="E2008" t="s">
-        <v>3155</v>
+        <v>3147</v>
       </c>
     </row>
     <row r="2009">
       <c r="A2009" t="s">
-        <v>3156</v>
+        <v>3148</v>
       </c>
       <c r="B2009" t="s">
-        <v>3156</v>
+        <v>3133</v>
       </c>
       <c r="C2009" t="s">
-        <v>3117</v>
+        <v>3149</v>
       </c>
       <c r="D2009" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E2009" t="s">
-        <v>3157</v>
+        <v>3150</v>
       </c>
     </row>
     <row r="2010">
       <c r="A2010" t="s">
-        <v>3156</v>
+        <v>3151</v>
       </c>
       <c r="B2010" t="s">
-        <v>3156</v>
+        <v>3149</v>
       </c>
       <c r="C2010" t="s">
-        <v>3121</v>
+        <v>1159</v>
       </c>
       <c r="D2010" t="s">
         <v>8</v>
       </c>
       <c r="E2010" t="s">
-        <v>3157</v>
+        <v>3152</v>
       </c>
     </row>
     <row r="2011">
       <c r="A2011" t="s">
-        <v>3158</v>
+        <v>3151</v>
       </c>
       <c r="B2011" t="s">
-        <v>3158</v>
+        <v>3149</v>
       </c>
       <c r="C2011" t="s">
-        <v>1146</v>
+        <v>2831</v>
       </c>
       <c r="D2011" t="s">
         <v>8</v>
       </c>
       <c r="E2011" t="s">
-        <v>3159</v>
+        <v>3152</v>
       </c>
     </row>
     <row r="2012">
       <c r="A2012" t="s">
-        <v>3160</v>
+        <v>3151</v>
       </c>
       <c r="B2012" t="s">
-        <v>3160</v>
+        <v>3149</v>
       </c>
       <c r="C2012" t="s">
-        <v>2499</v>
+        <v>1175</v>
       </c>
       <c r="D2012" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E2012" t="s">
-        <v>3161</v>
+        <v>3152</v>
       </c>
     </row>
     <row r="2013">
       <c r="A2013" t="s">
-        <v>3162</v>
+        <v>3151</v>
       </c>
       <c r="B2013" t="s">
-        <v>1820</v>
+        <v>3149</v>
       </c>
       <c r="C2013" t="s">
-        <v>1202</v>
+        <v>2834</v>
       </c>
       <c r="D2013" t="s">
         <v>8</v>
       </c>
       <c r="E2013" t="s">
-        <v>3163</v>
+        <v>3152</v>
       </c>
     </row>
     <row r="2014">
       <c r="A2014" t="s">
-        <v>3162</v>
+        <v>3153</v>
       </c>
       <c r="B2014" t="s">
-        <v>1820</v>
+        <v>2834</v>
       </c>
       <c r="C2014" t="s">
-        <v>1806</v>
+        <v>3154</v>
       </c>
       <c r="D2014" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E2014" t="s">
-        <v>3163</v>
+        <v>3155</v>
       </c>
     </row>
     <row r="2015">
       <c r="A2015" t="s">
-        <v>3164</v>
+        <v>3156</v>
       </c>
       <c r="B2015" t="s">
-        <v>64</v>
+        <v>3156</v>
       </c>
       <c r="C2015" t="s">
-        <v>421</v>
+        <v>3117</v>
       </c>
       <c r="D2015" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E2015" t="s">
-        <v>3165</v>
+        <v>3157</v>
       </c>
     </row>
     <row r="2016">
       <c r="A2016" t="s">
-        <v>3164</v>
+        <v>3156</v>
       </c>
       <c r="B2016" t="s">
-        <v>64</v>
+        <v>3156</v>
       </c>
       <c r="C2016" t="s">
-        <v>354</v>
+        <v>3121</v>
       </c>
       <c r="D2016" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E2016" t="s">
-        <v>3166</v>
+        <v>3157</v>
       </c>
     </row>
     <row r="2017">
       <c r="A2017" t="s">
-        <v>3167</v>
+        <v>3158</v>
       </c>
       <c r="B2017" t="s">
-        <v>3168</v>
+        <v>3158</v>
       </c>
       <c r="C2017" t="s">
-        <v>33</v>
+        <v>1146</v>
       </c>
       <c r="D2017" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E2017" t="s">
-        <v>3169</v>
+        <v>3159</v>
       </c>
     </row>
     <row r="2018">
       <c r="A2018" t="s">
-        <v>3170</v>
+        <v>3160</v>
       </c>
       <c r="B2018" t="s">
-        <v>3171</v>
+        <v>3160</v>
       </c>
       <c r="C2018" t="s">
-        <v>33</v>
+        <v>2499</v>
       </c>
       <c r="D2018" t="s">
         <v>13</v>
       </c>
       <c r="E2018" t="s">
-        <v>3172</v>
+        <v>3161</v>
       </c>
     </row>
     <row r="2019">
       <c r="A2019" t="s">
-        <v>3173</v>
+        <v>3162</v>
       </c>
       <c r="B2019" t="s">
-        <v>3174</v>
+        <v>1820</v>
       </c>
       <c r="C2019" t="s">
-        <v>505</v>
+        <v>1202</v>
       </c>
       <c r="D2019" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E2019" t="s">
-        <v>3175</v>
+        <v>3163</v>
       </c>
     </row>
     <row r="2020">
       <c r="A2020" t="s">
-        <v>1021</v>
+        <v>3162</v>
       </c>
       <c r="B2020" t="s">
-        <v>1021</v>
+        <v>1820</v>
       </c>
       <c r="C2020" t="s">
-        <v>113</v>
+        <v>1806</v>
       </c>
       <c r="D2020" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="E2020" t="s">
-        <v>3176</v>
+        <v>3163</v>
       </c>
     </row>
     <row r="2021">
       <c r="A2021" t="s">
-        <v>1021</v>
+        <v>3164</v>
       </c>
       <c r="B2021" t="s">
-        <v>1021</v>
+        <v>64</v>
       </c>
       <c r="C2021" t="s">
-        <v>117</v>
+        <v>421</v>
       </c>
       <c r="D2021" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E2021" t="s">
-        <v>3176</v>
+        <v>3165</v>
       </c>
     </row>
     <row r="2022">
       <c r="A2022" t="s">
-        <v>1021</v>
+        <v>3164</v>
       </c>
       <c r="B2022" t="s">
-        <v>1021</v>
+        <v>64</v>
       </c>
       <c r="C2022" t="s">
-        <v>119</v>
+        <v>354</v>
       </c>
       <c r="D2022" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E2022" t="s">
-        <v>3177</v>
+        <v>3166</v>
       </c>
     </row>
     <row r="2023">
       <c r="A2023" t="s">
-        <v>1021</v>
+        <v>3167</v>
       </c>
       <c r="B2023" t="s">
-        <v>1021</v>
+        <v>3168</v>
       </c>
       <c r="C2023" t="s">
-        <v>121</v>
+        <v>33</v>
       </c>
       <c r="D2023" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E2023" t="s">
-        <v>3176</v>
+        <v>3169</v>
       </c>
     </row>
     <row r="2024">
       <c r="A2024" t="s">
-        <v>1021</v>
+        <v>3170</v>
       </c>
       <c r="B2024" t="s">
-        <v>1021</v>
+        <v>3171</v>
       </c>
       <c r="C2024" t="s">
-        <v>481</v>
+        <v>33</v>
       </c>
       <c r="D2024" t="s">
         <v>13</v>
       </c>
       <c r="E2024" t="s">
-        <v>3176</v>
+        <v>3172</v>
       </c>
     </row>
     <row r="2025">
       <c r="A2025" t="s">
-        <v>3178</v>
+        <v>3173</v>
       </c>
       <c r="B2025" t="s">
-        <v>3178</v>
+        <v>3174</v>
       </c>
       <c r="C2025" t="s">
-        <v>1698</v>
+        <v>505</v>
       </c>
       <c r="D2025" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E2025" t="s">
-        <v>3179</v>
+        <v>3175</v>
       </c>
     </row>
     <row r="2026">
       <c r="A2026" t="s">
-        <v>3178</v>
+        <v>1021</v>
       </c>
       <c r="B2026" t="s">
-        <v>3178</v>
+        <v>1021</v>
       </c>
       <c r="C2026" t="s">
-        <v>1021</v>
+        <v>113</v>
       </c>
       <c r="D2026" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="E2026" t="s">
-        <v>3179</v>
+        <v>3176</v>
       </c>
     </row>
     <row r="2027">
       <c r="A2027" t="s">
-        <v>3180</v>
+        <v>1021</v>
       </c>
       <c r="B2027" t="s">
-        <v>3181</v>
+        <v>1021</v>
       </c>
       <c r="C2027" t="s">
-        <v>1021</v>
+        <v>117</v>
       </c>
       <c r="D2027" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="E2027" t="s">
-        <v>1702</v>
+        <v>3176</v>
       </c>
     </row>
     <row r="2028">
       <c r="A2028" t="s">
-        <v>3182</v>
+        <v>1021</v>
       </c>
       <c r="B2028" t="s">
-        <v>3183</v>
+        <v>1021</v>
       </c>
       <c r="C2028" t="s">
-        <v>53</v>
+        <v>119</v>
       </c>
       <c r="D2028" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="E2028" t="s">
-        <v>3184</v>
+        <v>3177</v>
       </c>
     </row>
     <row r="2029">
       <c r="A2029" t="s">
-        <v>3182</v>
+        <v>1021</v>
       </c>
       <c r="B2029" t="s">
-        <v>3183</v>
+        <v>1021</v>
       </c>
       <c r="C2029" t="s">
-        <v>16</v>
+        <v>121</v>
       </c>
       <c r="D2029" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="E2029" t="s">
-        <v>3185</v>
+        <v>3176</v>
       </c>
     </row>
     <row r="2030">
       <c r="A2030" t="s">
-        <v>3182</v>
+        <v>1021</v>
       </c>
       <c r="B2030" t="s">
-        <v>3183</v>
+        <v>1021</v>
       </c>
       <c r="C2030" t="s">
-        <v>2607</v>
+        <v>481</v>
       </c>
       <c r="D2030" t="s">
         <v>13</v>
       </c>
       <c r="E2030" t="s">
-        <v>3184</v>
+        <v>3176</v>
       </c>
     </row>
     <row r="2031">
       <c r="A2031" t="s">
-        <v>3182</v>
+        <v>3178</v>
       </c>
       <c r="B2031" t="s">
-        <v>3183</v>
+        <v>3178</v>
       </c>
       <c r="C2031" t="s">
-        <v>1170</v>
+        <v>1698</v>
       </c>
       <c r="D2031" t="s">
         <v>8</v>
       </c>
       <c r="E2031" t="s">
-        <v>3185</v>
+        <v>3179</v>
       </c>
     </row>
     <row r="2032">
       <c r="A2032" t="s">
-        <v>3182</v>
+        <v>3178</v>
       </c>
       <c r="B2032" t="s">
-        <v>3183</v>
+        <v>3178</v>
       </c>
       <c r="C2032" t="s">
-        <v>642</v>
+        <v>1021</v>
       </c>
       <c r="D2032" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E2032" t="s">
-        <v>3186</v>
+        <v>3179</v>
       </c>
     </row>
     <row r="2033">
       <c r="A2033" t="s">
-        <v>3187</v>
+        <v>3180</v>
       </c>
       <c r="B2033" t="s">
-        <v>64</v>
+        <v>3181</v>
       </c>
       <c r="C2033" t="s">
-        <v>172</v>
+        <v>1021</v>
       </c>
       <c r="D2033" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E2033" t="s">
-        <v>3188</v>
+        <v>1702</v>
       </c>
     </row>
     <row r="2034">
       <c r="A2034" t="s">
-        <v>3189</v>
+        <v>3182</v>
       </c>
       <c r="B2034" t="s">
-        <v>335</v>
+        <v>3183</v>
       </c>
       <c r="C2034" t="s">
-        <v>225</v>
+        <v>53</v>
       </c>
       <c r="D2034" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E2034" t="s">
-        <v>3190</v>
+        <v>3184</v>
       </c>
     </row>
     <row r="2035">
       <c r="A2035" t="s">
-        <v>3191</v>
+        <v>3182</v>
       </c>
       <c r="B2035" t="s">
-        <v>64</v>
+        <v>3183</v>
       </c>
       <c r="C2035" t="s">
-        <v>1021</v>
+        <v>16</v>
       </c>
       <c r="D2035" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E2035" t="s">
-        <v>3192</v>
+        <v>3185</v>
       </c>
     </row>
     <row r="2036">
       <c r="A2036" t="s">
-        <v>3193</v>
+        <v>3182</v>
       </c>
       <c r="B2036" t="s">
-        <v>3193</v>
+        <v>3183</v>
       </c>
       <c r="C2036" t="s">
-        <v>1946</v>
+        <v>2607</v>
       </c>
       <c r="D2036" t="s">
         <v>13</v>
       </c>
       <c r="E2036" t="s">
-        <v>3194</v>
+        <v>3184</v>
       </c>
     </row>
     <row r="2037">
       <c r="A2037" t="s">
-        <v>3193</v>
+        <v>3182</v>
       </c>
       <c r="B2037" t="s">
-        <v>3193</v>
+        <v>3183</v>
       </c>
       <c r="C2037" t="s">
-        <v>2078</v>
+        <v>1170</v>
       </c>
       <c r="D2037" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E2037" t="s">
-        <v>3195</v>
+        <v>3185</v>
       </c>
     </row>
     <row r="2038">
       <c r="A2038" t="s">
-        <v>3196</v>
+        <v>3182</v>
       </c>
       <c r="B2038" t="s">
-        <v>3196</v>
+        <v>3183</v>
       </c>
       <c r="C2038" t="s">
-        <v>2081</v>
+        <v>642</v>
       </c>
       <c r="D2038" t="s">
         <v>13</v>
       </c>
       <c r="E2038" t="s">
-        <v>3197</v>
+        <v>3186</v>
       </c>
     </row>
     <row r="2039">
       <c r="A2039" t="s">
-        <v>3198</v>
+        <v>3187</v>
       </c>
       <c r="B2039" t="s">
-        <v>1375</v>
+        <v>64</v>
       </c>
       <c r="C2039" t="s">
-        <v>285</v>
+        <v>172</v>
       </c>
       <c r="D2039" t="s">
         <v>13</v>
       </c>
       <c r="E2039" t="s">
-        <v>3199</v>
+        <v>3188</v>
       </c>
     </row>
     <row r="2040">
       <c r="A2040" t="s">
-        <v>3200</v>
+        <v>3189</v>
       </c>
       <c r="B2040" t="s">
-        <v>206</v>
+        <v>335</v>
       </c>
       <c r="C2040" t="s">
-        <v>347</v>
+        <v>225</v>
       </c>
       <c r="D2040" t="s">
         <v>13</v>
       </c>
       <c r="E2040" t="s">
-        <v>3201</v>
+        <v>3190</v>
       </c>
     </row>
     <row r="2041">
       <c r="A2041" t="s">
-        <v>3202</v>
+        <v>3191</v>
       </c>
       <c r="B2041" t="s">
-        <v>1375</v>
+        <v>64</v>
       </c>
       <c r="C2041" t="s">
-        <v>103</v>
+        <v>1021</v>
       </c>
       <c r="D2041" t="s">
         <v>13</v>
       </c>
       <c r="E2041" t="s">
-        <v>3203</v>
+        <v>3192</v>
       </c>
     </row>
     <row r="2042">
       <c r="A2042" t="s">
-        <v>3204</v>
+        <v>3193</v>
       </c>
       <c r="B2042" t="s">
-        <v>1310</v>
+        <v>3193</v>
       </c>
       <c r="C2042" t="s">
-        <v>29</v>
+        <v>1946</v>
       </c>
       <c r="D2042" t="s">
         <v>13</v>
       </c>
       <c r="E2042" t="s">
-        <v>3205</v>
+        <v>3194</v>
       </c>
     </row>
     <row r="2043">
       <c r="A2043" t="s">
-        <v>3206</v>
+        <v>3193</v>
       </c>
       <c r="B2043" t="s">
-        <v>3206</v>
+        <v>3193</v>
       </c>
       <c r="C2043" t="s">
-        <v>890</v>
+        <v>2078</v>
       </c>
       <c r="D2043" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E2043" t="s">
-        <v>3207</v>
+        <v>3195</v>
       </c>
     </row>
     <row r="2044">
       <c r="A2044" t="s">
-        <v>3206</v>
+        <v>3196</v>
       </c>
       <c r="B2044" t="s">
-        <v>3208</v>
+        <v>3196</v>
       </c>
       <c r="C2044" t="s">
-        <v>373</v>
+        <v>2081</v>
       </c>
       <c r="D2044" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E2044" t="s">
-        <v>732</v>
+        <v>3197</v>
       </c>
     </row>
     <row r="2045">
       <c r="A2045" t="s">
-        <v>3209</v>
+        <v>3198</v>
       </c>
       <c r="B2045" t="s">
-        <v>3210</v>
+        <v>1375</v>
       </c>
       <c r="C2045" t="s">
-        <v>3211</v>
+        <v>285</v>
       </c>
       <c r="D2045" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E2045" t="s">
-        <v>3212</v>
+        <v>3199</v>
       </c>
     </row>
     <row r="2046">
       <c r="A2046" t="s">
-        <v>2265</v>
+        <v>3200</v>
       </c>
       <c r="B2046" t="s">
-        <v>2265</v>
+        <v>206</v>
       </c>
       <c r="C2046" t="s">
-        <v>3211</v>
+        <v>347</v>
       </c>
       <c r="D2046" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E2046" t="s">
-        <v>3213</v>
+        <v>3201</v>
       </c>
     </row>
     <row r="2047">
       <c r="A2047" t="s">
-        <v>2265</v>
+        <v>3202</v>
       </c>
       <c r="B2047" t="s">
-        <v>3214</v>
+        <v>1375</v>
       </c>
       <c r="C2047" t="s">
-        <v>2265</v>
+        <v>103</v>
       </c>
       <c r="D2047" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E2047" t="s">
-        <v>3215</v>
+        <v>3203</v>
       </c>
     </row>
     <row r="2048">
       <c r="A2048" t="s">
-        <v>3216</v>
+        <v>3204</v>
       </c>
       <c r="B2048" t="s">
-        <v>3217</v>
+        <v>1310</v>
       </c>
       <c r="C2048" t="s">
-        <v>159</v>
+        <v>29</v>
       </c>
       <c r="D2048" t="s">
         <v>13</v>
       </c>
       <c r="E2048" t="s">
-        <v>3218</v>
+        <v>3205</v>
       </c>
     </row>
     <row r="2049">
       <c r="A2049" t="s">
-        <v>3219</v>
+        <v>3206</v>
       </c>
       <c r="B2049" t="s">
-        <v>3219</v>
+        <v>3206</v>
       </c>
       <c r="C2049" t="s">
-        <v>399</v>
+        <v>890</v>
       </c>
       <c r="D2049" t="s">
         <v>8</v>
       </c>
       <c r="E2049" t="s">
-        <v>3220</v>
+        <v>3207</v>
       </c>
     </row>
     <row r="2050">
       <c r="A2050" t="s">
-        <v>3219</v>
+        <v>3206</v>
       </c>
       <c r="B2050" t="s">
-        <v>3219</v>
+        <v>3208</v>
       </c>
       <c r="C2050" t="s">
-        <v>401</v>
+        <v>373</v>
       </c>
       <c r="D2050" t="s">
         <v>8</v>
       </c>
       <c r="E2050" t="s">
-        <v>3221</v>
+        <v>732</v>
       </c>
     </row>
     <row r="2051">
       <c r="A2051" t="s">
-        <v>3219</v>
+        <v>3209</v>
       </c>
       <c r="B2051" t="s">
-        <v>3219</v>
+        <v>3210</v>
       </c>
       <c r="C2051" t="s">
-        <v>53</v>
+        <v>3211</v>
       </c>
       <c r="D2051" t="s">
         <v>8</v>
       </c>
       <c r="E2051" t="s">
-        <v>3222</v>
+        <v>3212</v>
       </c>
     </row>
     <row r="2052">
       <c r="A2052" t="s">
-        <v>3223</v>
+        <v>2265</v>
       </c>
       <c r="B2052" t="s">
-        <v>3223</v>
+        <v>2265</v>
       </c>
       <c r="C2052" t="s">
-        <v>162</v>
+        <v>3211</v>
       </c>
       <c r="D2052" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E2052" t="s">
-        <v>3224</v>
+        <v>3213</v>
       </c>
     </row>
     <row r="2053">
       <c r="A2053" t="s">
-        <v>3225</v>
+        <v>2265</v>
       </c>
       <c r="B2053" t="s">
-        <v>222</v>
+        <v>3214</v>
       </c>
       <c r="C2053" t="s">
-        <v>575</v>
+        <v>2265</v>
       </c>
       <c r="D2053" t="s">
         <v>8</v>
       </c>
       <c r="E2053" t="s">
-        <v>3226</v>
+        <v>3215</v>
       </c>
     </row>
     <row r="2054">
       <c r="A2054" t="s">
-        <v>3227</v>
+        <v>3216</v>
       </c>
       <c r="B2054" t="s">
-        <v>357</v>
+        <v>3217</v>
       </c>
       <c r="C2054" t="s">
-        <v>841</v>
+        <v>159</v>
       </c>
       <c r="D2054" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E2054" t="s">
-        <v>3228</v>
+        <v>3218</v>
       </c>
     </row>
     <row r="2055">
       <c r="A2055" t="s">
-        <v>3229</v>
+        <v>3219</v>
       </c>
       <c r="B2055" t="s">
-        <v>211</v>
+        <v>3219</v>
       </c>
       <c r="C2055" t="s">
-        <v>693</v>
+        <v>399</v>
       </c>
       <c r="D2055" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E2055" t="s">
-        <v>3230</v>
+        <v>3220</v>
       </c>
     </row>
     <row r="2056">
       <c r="A2056" t="s">
-        <v>3231</v>
+        <v>3219</v>
       </c>
       <c r="B2056" t="s">
-        <v>211</v>
+        <v>3219</v>
       </c>
       <c r="C2056" t="s">
-        <v>693</v>
+        <v>401</v>
       </c>
       <c r="D2056" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E2056" t="s">
-        <v>3232</v>
+        <v>3221</v>
       </c>
     </row>
     <row r="2057">
       <c r="A2057" t="s">
-        <v>3233</v>
+        <v>3219</v>
       </c>
       <c r="B2057" t="s">
-        <v>335</v>
+        <v>3219</v>
       </c>
       <c r="C2057" t="s">
-        <v>2753</v>
+        <v>53</v>
       </c>
       <c r="D2057" t="s">
         <v>8</v>
       </c>
       <c r="E2057" t="s">
-        <v>3234</v>
+        <v>3222</v>
       </c>
     </row>
     <row r="2058">
       <c r="A2058" t="s">
-        <v>3233</v>
+        <v>3223</v>
       </c>
       <c r="B2058" t="s">
-        <v>335</v>
+        <v>3223</v>
       </c>
       <c r="C2058" t="s">
-        <v>3026</v>
+        <v>162</v>
       </c>
       <c r="D2058" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E2058" t="s">
-        <v>3234</v>
+        <v>3224</v>
       </c>
     </row>
     <row r="2059">
       <c r="A2059" t="s">
-        <v>3235</v>
+        <v>3225</v>
       </c>
       <c r="B2059" t="s">
-        <v>3236</v>
+        <v>222</v>
       </c>
       <c r="C2059" t="s">
-        <v>2753</v>
+        <v>575</v>
       </c>
       <c r="D2059" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E2059" t="s">
-        <v>3237</v>
+        <v>3226</v>
       </c>
     </row>
     <row r="2060">
       <c r="A2060" t="s">
-        <v>3238</v>
+        <v>3227</v>
       </c>
       <c r="B2060" t="s">
-        <v>3239</v>
+        <v>357</v>
       </c>
       <c r="C2060" t="s">
-        <v>2753</v>
+        <v>841</v>
       </c>
       <c r="D2060" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E2060" t="s">
-        <v>3240</v>
+        <v>3228</v>
       </c>
     </row>
     <row r="2061">
       <c r="A2061" t="s">
-        <v>3241</v>
+        <v>3229</v>
       </c>
       <c r="B2061" t="s">
-        <v>3242</v>
+        <v>211</v>
       </c>
       <c r="C2061" t="s">
-        <v>492</v>
+        <v>693</v>
       </c>
       <c r="D2061" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E2061" t="s">
-        <v>3243</v>
+        <v>3230</v>
       </c>
     </row>
     <row r="2062">
       <c r="A2062" t="s">
-        <v>3244</v>
+        <v>3231</v>
       </c>
       <c r="B2062" t="s">
-        <v>3245</v>
+        <v>211</v>
       </c>
       <c r="C2062" t="s">
-        <v>492</v>
+        <v>693</v>
       </c>
       <c r="D2062" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E2062" t="s">
-        <v>3246</v>
+        <v>3232</v>
       </c>
     </row>
     <row r="2063">
       <c r="A2063" t="s">
-        <v>3247</v>
+        <v>3233</v>
       </c>
       <c r="B2063" t="s">
-        <v>3248</v>
+        <v>335</v>
       </c>
       <c r="C2063" t="s">
-        <v>117</v>
+        <v>2753</v>
       </c>
       <c r="D2063" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="E2063" t="s">
-        <v>3249</v>
+        <v>3234</v>
       </c>
     </row>
     <row r="2064">
       <c r="A2064" t="s">
-        <v>3247</v>
+        <v>3233</v>
       </c>
       <c r="B2064" t="s">
-        <v>3248</v>
+        <v>335</v>
       </c>
       <c r="C2064" t="s">
-        <v>121</v>
+        <v>3026</v>
       </c>
       <c r="D2064" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="E2064" t="s">
-        <v>3250</v>
+        <v>3234</v>
       </c>
     </row>
     <row r="2065">
       <c r="A2065" t="s">
-        <v>291</v>
+        <v>3235</v>
       </c>
       <c r="B2065" t="s">
-        <v>291</v>
+        <v>3236</v>
       </c>
       <c r="C2065" t="s">
-        <v>35</v>
+        <v>2753</v>
       </c>
       <c r="D2065" t="s">
         <v>13</v>
       </c>
       <c r="E2065" t="s">
-        <v>3251</v>
+        <v>3237</v>
       </c>
     </row>
     <row r="2066">
       <c r="A2066" t="s">
-        <v>291</v>
+        <v>3238</v>
       </c>
       <c r="B2066" t="s">
-        <v>291</v>
+        <v>3239</v>
       </c>
       <c r="C2066" t="s">
-        <v>373</v>
+        <v>2753</v>
       </c>
       <c r="D2066" t="s">
         <v>13</v>
       </c>
       <c r="E2066" t="s">
-        <v>3252</v>
+        <v>3240</v>
       </c>
     </row>
     <row r="2067">
       <c r="A2067" t="s">
-        <v>291</v>
+        <v>3241</v>
       </c>
       <c r="B2067" t="s">
-        <v>291</v>
+        <v>3242</v>
       </c>
       <c r="C2067" t="s">
-        <v>911</v>
+        <v>492</v>
       </c>
       <c r="D2067" t="s">
         <v>17</v>
       </c>
       <c r="E2067" t="s">
-        <v>3253</v>
+        <v>3243</v>
       </c>
     </row>
     <row r="2068">
       <c r="A2068" t="s">
-        <v>3254</v>
+        <v>3244</v>
       </c>
       <c r="B2068" t="s">
-        <v>211</v>
+        <v>3245</v>
       </c>
       <c r="C2068" t="s">
-        <v>735</v>
+        <v>492</v>
       </c>
       <c r="D2068" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E2068" t="s">
-        <v>3255</v>
+        <v>3246</v>
       </c>
     </row>
     <row r="2069">
       <c r="A2069" t="s">
-        <v>3256</v>
+        <v>3247</v>
       </c>
       <c r="B2069" t="s">
-        <v>211</v>
+        <v>3248</v>
       </c>
       <c r="C2069" t="s">
-        <v>735</v>
+        <v>117</v>
       </c>
       <c r="D2069" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E2069" t="s">
-        <v>3257</v>
+        <v>3249</v>
       </c>
     </row>
     <row r="2070">
       <c r="A2070" t="s">
-        <v>3258</v>
+        <v>3247</v>
       </c>
       <c r="B2070" t="s">
-        <v>211</v>
+        <v>3248</v>
       </c>
       <c r="C2070" t="s">
-        <v>735</v>
+        <v>121</v>
       </c>
       <c r="D2070" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E2070" t="s">
-        <v>3259</v>
+        <v>3250</v>
       </c>
     </row>
     <row r="2071">
       <c r="A2071" t="s">
-        <v>3260</v>
+        <v>291</v>
       </c>
       <c r="B2071" t="s">
         <v>291</v>
       </c>
       <c r="C2071" t="s">
-        <v>103</v>
+        <v>35</v>
       </c>
       <c r="D2071" t="s">
         <v>13</v>
       </c>
       <c r="E2071" t="s">
-        <v>3261</v>
+        <v>3251</v>
       </c>
     </row>
     <row r="2072">
       <c r="A2072" t="s">
-        <v>3262</v>
+        <v>291</v>
       </c>
       <c r="B2072" t="s">
-        <v>3262</v>
+        <v>291</v>
       </c>
       <c r="C2072" t="s">
-        <v>1935</v>
+        <v>373</v>
       </c>
       <c r="D2072" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E2072" t="s">
-        <v>3263</v>
+        <v>3252</v>
       </c>
     </row>
     <row r="2073">
       <c r="A2073" t="s">
-        <v>3262</v>
+        <v>291</v>
       </c>
       <c r="B2073" t="s">
-        <v>3262</v>
+        <v>291</v>
       </c>
       <c r="C2073" t="s">
-        <v>922</v>
+        <v>911</v>
       </c>
       <c r="D2073" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="E2073" t="s">
-        <v>3263</v>
+        <v>3253</v>
       </c>
     </row>
     <row r="2074">
       <c r="A2074" t="s">
-        <v>3264</v>
+        <v>3254</v>
       </c>
       <c r="B2074" t="s">
-        <v>3265</v>
+        <v>211</v>
       </c>
       <c r="C2074" t="s">
-        <v>373</v>
+        <v>735</v>
       </c>
       <c r="D2074" t="s">
         <v>13</v>
       </c>
       <c r="E2074" t="s">
-        <v>3266</v>
+        <v>3255</v>
       </c>
     </row>
     <row r="2075">
       <c r="A2075" t="s">
-        <v>3264</v>
+        <v>3256</v>
       </c>
       <c r="B2075" t="s">
-        <v>3267</v>
+        <v>211</v>
       </c>
       <c r="C2075" t="s">
-        <v>103</v>
+        <v>735</v>
       </c>
       <c r="D2075" t="s">
         <v>13</v>
       </c>
       <c r="E2075" t="s">
-        <v>3266</v>
+        <v>3257</v>
       </c>
     </row>
     <row r="2076">
       <c r="A2076" t="s">
-        <v>3268</v>
+        <v>3258</v>
       </c>
       <c r="B2076" t="s">
-        <v>3269</v>
+        <v>211</v>
       </c>
       <c r="C2076" t="s">
-        <v>555</v>
+        <v>735</v>
       </c>
       <c r="D2076" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E2076" t="s">
-        <v>3270</v>
+        <v>3259</v>
       </c>
     </row>
     <row r="2077">
       <c r="A2077" t="s">
-        <v>3271</v>
+        <v>3260</v>
       </c>
       <c r="B2077" t="s">
-        <v>3272</v>
+        <v>291</v>
       </c>
       <c r="C2077" t="s">
-        <v>455</v>
+        <v>103</v>
       </c>
       <c r="D2077" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E2077" t="s">
-        <v>3273</v>
+        <v>3261</v>
       </c>
     </row>
     <row r="2078">
       <c r="A2078" t="s">
-        <v>3271</v>
+        <v>3262</v>
       </c>
       <c r="B2078" t="s">
-        <v>3272</v>
+        <v>3262</v>
       </c>
       <c r="C2078" t="s">
-        <v>458</v>
+        <v>1935</v>
       </c>
       <c r="D2078" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="E2078" t="s">
-        <v>3274</v>
+        <v>3263</v>
       </c>
     </row>
     <row r="2079">
       <c r="A2079" t="s">
-        <v>3275</v>
+        <v>3262</v>
       </c>
       <c r="B2079" t="s">
-        <v>291</v>
+        <v>3262</v>
       </c>
       <c r="C2079" t="s">
-        <v>115</v>
+        <v>922</v>
       </c>
       <c r="D2079" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E2079" t="s">
-        <v>3276</v>
+        <v>3263</v>
       </c>
     </row>
     <row r="2080">
       <c r="A2080" t="s">
-        <v>3277</v>
+        <v>3264</v>
       </c>
       <c r="B2080" t="s">
-        <v>3277</v>
+        <v>3265</v>
       </c>
       <c r="C2080" t="s">
-        <v>399</v>
+        <v>373</v>
       </c>
       <c r="D2080" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E2080" t="s">
-        <v>3278</v>
+        <v>3266</v>
       </c>
     </row>
     <row r="2081">
       <c r="A2081" t="s">
-        <v>3277</v>
+        <v>3264</v>
       </c>
       <c r="B2081" t="s">
-        <v>3277</v>
+        <v>3267</v>
       </c>
       <c r="C2081" t="s">
-        <v>49</v>
+        <v>103</v>
       </c>
       <c r="D2081" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E2081" t="s">
-        <v>3278</v>
+        <v>3266</v>
       </c>
     </row>
     <row r="2082">
       <c r="A2082" t="s">
-        <v>3279</v>
+        <v>3268</v>
       </c>
       <c r="B2082" t="s">
-        <v>191</v>
+        <v>3269</v>
       </c>
       <c r="C2082" t="s">
-        <v>57</v>
+        <v>555</v>
       </c>
       <c r="D2082" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E2082" t="s">
-        <v>3280</v>
+        <v>3270</v>
       </c>
     </row>
     <row r="2083">
       <c r="A2083" t="s">
-        <v>3281</v>
+        <v>3271</v>
       </c>
       <c r="B2083" t="s">
-        <v>191</v>
+        <v>3272</v>
       </c>
       <c r="C2083" t="s">
-        <v>31</v>
+        <v>455</v>
       </c>
       <c r="D2083" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E2083" t="s">
-        <v>3282</v>
+        <v>3273</v>
       </c>
     </row>
     <row r="2084">
       <c r="A2084" t="s">
-        <v>3281</v>
+        <v>3271</v>
       </c>
       <c r="B2084" t="s">
-        <v>191</v>
+        <v>3272</v>
       </c>
       <c r="C2084" t="s">
-        <v>799</v>
+        <v>458</v>
       </c>
       <c r="D2084" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E2084" t="s">
-        <v>3283</v>
+        <v>3274</v>
       </c>
     </row>
     <row r="2085">
       <c r="A2085" t="s">
-        <v>3284</v>
+        <v>3275</v>
       </c>
       <c r="B2085" t="s">
-        <v>3285</v>
+        <v>291</v>
       </c>
       <c r="C2085" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D2085" t="s">
         <v>13</v>
       </c>
       <c r="E2085" t="s">
-        <v>3286</v>
+        <v>3276</v>
       </c>
     </row>
     <row r="2086">
       <c r="A2086" t="s">
-        <v>3287</v>
+        <v>3277</v>
       </c>
       <c r="B2086" t="s">
-        <v>3285</v>
+        <v>3277</v>
       </c>
       <c r="C2086" t="s">
-        <v>117</v>
+        <v>399</v>
       </c>
       <c r="D2086" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E2086" t="s">
-        <v>3288</v>
+        <v>3278</v>
       </c>
     </row>
     <row r="2087">
       <c r="A2087" t="s">
+        <v>3277</v>
+      </c>
+      <c r="B2087" t="s">
+        <v>3277</v>
+      </c>
+      <c r="C2087" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2087" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2087" t="s">
+        <v>3278</v>
+      </c>
+    </row>
+    <row r="2088">
+      <c r="A2088" t="s">
+        <v>3279</v>
+      </c>
+      <c r="B2088" t="s">
+        <v>191</v>
+      </c>
+      <c r="C2088" t="s">
+        <v>57</v>
+      </c>
+      <c r="D2088" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2088" t="s">
+        <v>3280</v>
+      </c>
+    </row>
+    <row r="2089">
+      <c r="A2089" t="s">
+        <v>3281</v>
+      </c>
+      <c r="B2089" t="s">
+        <v>191</v>
+      </c>
+      <c r="C2089" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2089" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2089" t="s">
+        <v>3282</v>
+      </c>
+    </row>
+    <row r="2090">
+      <c r="A2090" t="s">
+        <v>3281</v>
+      </c>
+      <c r="B2090" t="s">
+        <v>191</v>
+      </c>
+      <c r="C2090" t="s">
+        <v>799</v>
+      </c>
+      <c r="D2090" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2090" t="s">
+        <v>3283</v>
+      </c>
+    </row>
+    <row r="2091">
+      <c r="A2091" t="s">
+        <v>3284</v>
+      </c>
+      <c r="B2091" t="s">
+        <v>3285</v>
+      </c>
+      <c r="C2091" t="s">
+        <v>117</v>
+      </c>
+      <c r="D2091" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2091" t="s">
+        <v>3286</v>
+      </c>
+    </row>
+    <row r="2092">
+      <c r="A2092" t="s">
+        <v>3287</v>
+      </c>
+      <c r="B2092" t="s">
+        <v>3285</v>
+      </c>
+      <c r="C2092" t="s">
+        <v>117</v>
+      </c>
+      <c r="D2092" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2092" t="s">
+        <v>3288</v>
+      </c>
+    </row>
+    <row r="2093">
+      <c r="A2093" t="s">
         <v>3289</v>
       </c>
-      <c r="B2087" t="s">
+      <c r="B2093" t="s">
         <v>2118</v>
       </c>
-      <c r="C2087" t="s">
+      <c r="C2093" t="s">
         <v>378</v>
       </c>
-      <c r="D2087" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2087" t="s">
+      <c r="D2093" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2093" t="s">
         <v>3290</v>
       </c>
     </row>

</xml_diff>